<commit_message>
Restore Config boolean cells to literals after recalculation
LibreOffice's round-trip rewrites boolean cells as =TRUE()/=FALSE()
formulas. They evaluate correctly and the VBA reads them fine, but these
are cells the operator is told to edit, and a formula sitting in a yellow
input cell is a trap: editing it replaces a formula rather than a value,
and the formula bar shows TRUE() where a plain TRUE belongs.

phase2 now coerces them back to literals after the recalculation pass, so
Config carries only its three intended commission formulas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HHvxabz67VZkmriPMTpFvX
</commit_message>
<xml_diff>
--- a/TT_ZScore_Monitor.xlsx
+++ b/TT_ZScore_Monitor.xlsx
@@ -1040,7 +1040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:Q84"/>
+  <dimension ref="A1:Q84"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="64" min="1" max="1"/>
@@ -1562,6 +1562,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="15" customHeight="1" s="65">
       <c r="B17" s="80" t="inlineStr">
         <is>
@@ -1733,6 +1734,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26" ht="15" customHeight="1" s="65">
       <c r="B26" s="79" t="inlineStr">
         <is>
@@ -2345,6 +2347,7 @@
       <c r="F68" s="85" t="n"/>
       <c r="G68" s="85" t="n"/>
     </row>
+    <row r="69"/>
     <row r="70" ht="15" customHeight="1" s="65">
       <c r="B70" s="90" t="inlineStr">
         <is>
@@ -2429,6 +2432,7 @@
         </is>
       </c>
     </row>
+    <row r="82"/>
     <row r="83" ht="15" customHeight="1" s="65">
       <c r="B83" s="103" t="inlineStr">
         <is>
@@ -2560,6 +2564,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="15" customHeight="1" s="65">
       <c r="A7" s="105" t="inlineStr">
         <is>
@@ -2834,13 +2839,11 @@
           <t>TICK_ARCHIVE_ENABLED</t>
         </is>
       </c>
-      <c r="B19" s="76">
-        <f>TRUE()</f>
-        <v/>
-      </c>
-      <c r="C19" s="84">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B19" s="76" t="b">
+        <v>1</v>
+      </c>
+      <c r="C19" s="84" t="b">
+        <v>1</v>
       </c>
       <c r="D19" s="84" t="inlineStr">
         <is>
@@ -2895,6 +2898,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="65">
       <c r="A23" s="105" t="inlineStr">
         <is>
@@ -3071,6 +3075,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32" ht="15" customHeight="1" s="65">
       <c r="A32" s="105" t="inlineStr">
         <is>
@@ -3178,6 +3183,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38" ht="15" customHeight="1" s="65">
       <c r="A38" s="105" t="inlineStr">
         <is>
@@ -3354,6 +3360,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="65">
       <c r="A47" s="105" t="inlineStr">
         <is>
@@ -3398,13 +3405,11 @@
           <t>ALERT_ENABLED</t>
         </is>
       </c>
-      <c r="B49" s="76">
-        <f>TRUE()</f>
-        <v/>
-      </c>
-      <c r="C49" s="84">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B49" s="76" t="b">
+        <v>1</v>
+      </c>
+      <c r="C49" s="84" t="b">
+        <v>1</v>
       </c>
       <c r="D49" s="84" t="inlineStr">
         <is>
@@ -3523,13 +3528,11 @@
           <t>ALERT_ONLY_IF_EDGE_PASSES</t>
         </is>
       </c>
-      <c r="B54" s="76">
-        <f>TRUE()</f>
-        <v/>
-      </c>
-      <c r="C54" s="84">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B54" s="76" t="b">
+        <v>1</v>
+      </c>
+      <c r="C54" s="84" t="b">
+        <v>1</v>
       </c>
       <c r="D54" s="84" t="inlineStr">
         <is>
@@ -3548,13 +3551,11 @@
           <t>ALERT_SPEAK</t>
         </is>
       </c>
-      <c r="B55" s="76">
-        <f>FALSE()</f>
-        <v/>
-      </c>
-      <c r="C55" s="84">
-        <f>FALSE()</f>
-        <v/>
+      <c r="B55" s="76" t="b">
+        <v>0</v>
+      </c>
+      <c r="C55" s="84" t="b">
+        <v>0</v>
       </c>
       <c r="D55" s="84" t="inlineStr">
         <is>
@@ -3567,6 +3568,7 @@
         </is>
       </c>
     </row>
+    <row r="56"/>
     <row r="57" ht="15" customHeight="1" s="65">
       <c r="A57" s="105" t="inlineStr">
         <is>
@@ -3611,13 +3613,11 @@
           <t>WARM_START_ENABLED</t>
         </is>
       </c>
-      <c r="B59" s="76">
-        <f>TRUE()</f>
-        <v/>
-      </c>
-      <c r="C59" s="84">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B59" s="76" t="b">
+        <v>1</v>
+      </c>
+      <c r="C59" s="84" t="b">
+        <v>1</v>
       </c>
       <c r="D59" s="84" t="inlineStr">
         <is>
@@ -3659,13 +3659,11 @@
           <t>LOG_ENABLED</t>
         </is>
       </c>
-      <c r="B61" s="76">
-        <f>TRUE()</f>
-        <v/>
-      </c>
-      <c r="C61" s="84">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B61" s="76" t="b">
+        <v>1</v>
+      </c>
+      <c r="C61" s="84" t="b">
+        <v>1</v>
       </c>
       <c r="D61" s="84" t="inlineStr">
         <is>
@@ -3701,6 +3699,7 @@
         </is>
       </c>
     </row>
+    <row r="63"/>
     <row r="64" ht="15" customHeight="1" s="65">
       <c r="A64" s="105" t="inlineStr">
         <is>
@@ -3809,6 +3808,7 @@
         </is>
       </c>
     </row>
+    <row r="70"/>
     <row r="71" ht="15" customHeight="1" s="65">
       <c r="A71" s="105" t="inlineStr">
         <is>
@@ -3896,9 +3896,8 @@
           <t>SPREAD_1</t>
         </is>
       </c>
-      <c r="B74" s="76">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B74" s="76" t="b">
+        <v>1</v>
       </c>
       <c r="C74" s="108" t="inlineStr">
         <is>
@@ -3942,9 +3941,8 @@
           <t>SPREAD_2</t>
         </is>
       </c>
-      <c r="B75" s="76">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B75" s="76" t="b">
+        <v>1</v>
       </c>
       <c r="C75" s="108" t="inlineStr">
         <is>
@@ -3988,9 +3986,8 @@
           <t>SPREAD_3</t>
         </is>
       </c>
-      <c r="B76" s="76">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B76" s="76" t="b">
+        <v>1</v>
       </c>
       <c r="C76" s="108" t="inlineStr">
         <is>
@@ -4034,9 +4031,8 @@
           <t>SPREAD_4</t>
         </is>
       </c>
-      <c r="B77" s="76">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B77" s="76" t="b">
+        <v>1</v>
       </c>
       <c r="C77" s="108" t="inlineStr">
         <is>
@@ -4074,6 +4070,7 @@
         </is>
       </c>
     </row>
+    <row r="78"/>
     <row r="79" ht="15" customHeight="1" s="65">
       <c r="A79" s="116" t="inlineStr">
         <is>
@@ -4142,6 +4139,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="65">
       <c r="A5" s="119" t="inlineStr">
         <is>
@@ -4424,6 +4422,9 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="65">
       <c r="A15" s="119" t="inlineStr">
         <is>
@@ -4596,6 +4597,8 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
+    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="65">
       <c r="A23" s="122" t="inlineStr">
         <is>
@@ -4847,6 +4850,7 @@
         <v/>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="15" customHeight="1" s="65">
       <c r="A34" s="122" t="inlineStr">
         <is>
@@ -4921,6 +4925,7 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41" ht="15" customHeight="1" s="65">
       <c r="A41" s="67" t="inlineStr">
         <is>
@@ -5300,7 +5305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:G39"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="64" min="1" max="1"/>
@@ -5316,6 +5321,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1" s="65">
       <c r="B3" s="124" t="inlineStr">
         <is>
@@ -5372,6 +5378,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="65">
       <c r="B12" s="80" t="inlineStr">
         <is>
@@ -5421,6 +5428,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="65">
       <c r="B20" s="80" t="inlineStr">
         <is>
@@ -5453,6 +5461,7 @@
         <v>0.02</v>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="22.35" customHeight="1" s="65">
       <c r="B24" s="79" t="inlineStr">
         <is>
@@ -5526,6 +5535,7 @@
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="15" customHeight="1" s="65">
       <c r="B28" s="67" t="inlineStr">
         <is>
@@ -5540,6 +5550,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="15" customHeight="1" s="65">
       <c r="B31" s="80" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Set WIN_PCT to 0.004, targeting ~1.25 sigma
At 0.01 the take-profit landed 2.95 sigma out on HO/CL and 2.79 on the
3:2:1 - past the mean when entering at ENTRY_Z 2.5, so both needed an
overshoot rather than the reversion the z measured. 0.004 puts all three
legged spreads at 1.1-1.4 sigma, inside the mean, and matches the
0.5 x |z| x sigma capture the edge filter already assumes.

Derived from a single ~2h window (sigma 0.3598 / 0.0684 / 0.2392 against
costs of 110.04 / 47.64 / 254.52), so it is a starting point, not a
calibrated value - re-derive once sigma has been measured properly.

TP-in-sigma is invariant to LOTS: cost and win both scale linearly, so
the lots cancel. LOTS stays purely a position-sizing decision.
</commit_message>
<xml_diff>
--- a/TT_ZScore_Monitor.xlsx
+++ b/TT_ZScore_Monitor.xlsx
@@ -4665,10 +4665,10 @@
         </is>
       </c>
       <c r="B43" s="263" t="n">
-        <v>0.01</v>
+        <v>0.004</v>
       </c>
       <c r="C43" s="264" t="n">
-        <v>0.01</v>
+        <v>0.004</v>
       </c>
       <c r="D43" s="239" t="inlineStr">
         <is>
@@ -4677,7 +4677,7 @@
       </c>
       <c r="E43" s="261" t="inlineStr">
         <is>
-          <t>Percentage win, as a FRACTION - 0.01 is 1%, 0.02 is 2%. Used only when TP_MODE = PCT_NOTIONAL.</t>
+          <t>Percentage win, as a FRACTION - 0.01 is 1%, 0.004 is 0.4%. Used only when TP_MODE = PCT_NOTIONAL. 0.004 targets about 1.25 sigma, the same capture the edge filter assumes at ENTRY_Z, which keeps the take-profit inside the mean on all three legged spreads. Re-derive it once sigma has been measured over more than a single window.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roll CL and BZ to the November series; warn about the shared CL leg
Brent October expired, so BZ - CL went dark. INSTRUMENT_3 and INSTRUMENT_4
now ship as CLX6 and BZX6.

CL is a leg of all three spreads, so rolling it alone leaves the cracks as
October RBOB and ULSD against November WTI - a crack plus a calendar spread,
which is not what the z-score measured. Config now says so beside the table.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HHvxabz67VZkmriPMTpFvX
</commit_message>
<xml_diff>
--- a/TT_ZScore_Monitor.xlsx
+++ b/TT_ZScore_Monitor.xlsx
@@ -3881,7 +3881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K103"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="141" min="1" max="1"/>
@@ -5340,292 +5340,254 @@
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="143">
-      <c r="A80" s="256" t="inlineStr">
+      <c r="A80" s="252" t="inlineStr">
+        <is>
+          <t>CL is a leg of ALL THREE spreads. Moving it to November while RBOB and ULSD stay in October turns the cracks into a crack PLUS a calendar spread - not the thing the z-score was measuring. Roll RBOB and ULSD with it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="15" customHeight="1" s="143">
+      <c r="A81" s="256" t="inlineStr">
         <is>
           <t>Slot</t>
         </is>
       </c>
-      <c r="B80" s="256" t="inlineStr">
+      <c r="B81" s="256" t="inlineStr">
         <is>
           <t>TT short name</t>
         </is>
       </c>
-      <c r="C80" s="256" t="inlineStr">
+      <c r="C81" s="256" t="inlineStr">
         <is>
           <t>Instrument</t>
         </is>
       </c>
-      <c r="D80" s="256" t="n"/>
-      <c r="E80" s="256" t="inlineStr">
+      <c r="D81" s="256" t="n"/>
+      <c r="E81" s="256" t="inlineStr">
         <is>
           <t>Used as</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="15" customHeight="1" s="143">
-      <c r="A81" s="249" t="inlineStr">
-        <is>
-          <t>INSTRUMENT_1</t>
-        </is>
-      </c>
-      <c r="B81" s="259" t="inlineStr">
-        <is>
-          <t>RBV6</t>
-        </is>
-      </c>
-      <c r="C81" s="235" t="inlineStr">
-        <is>
-          <t>RBOB Gasoline</t>
-        </is>
-      </c>
-      <c r="E81" s="264" t="inlineStr">
-        <is>
-          <t>leg of the 3:2:1</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="143">
       <c r="A82" s="249" t="inlineStr">
         <is>
-          <t>INSTRUMENT_2</t>
+          <t>INSTRUMENT_1</t>
         </is>
       </c>
       <c r="B82" s="259" t="inlineStr">
         <is>
-          <t>HOV6</t>
+          <t>RBV6</t>
         </is>
       </c>
       <c r="C82" s="235" t="inlineStr">
         <is>
-          <t>NY Harbor ULSD</t>
+          <t>RBOB Gasoline</t>
         </is>
       </c>
       <c r="E82" s="264" t="inlineStr">
         <is>
-          <t>leg of HO/CL and the 3:2:1</t>
+          <t>leg of the 3:2:1</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="143">
       <c r="A83" s="249" t="inlineStr">
         <is>
-          <t>INSTRUMENT_3</t>
+          <t>INSTRUMENT_2</t>
         </is>
       </c>
       <c r="B83" s="259" t="inlineStr">
         <is>
-          <t>CLV6</t>
+          <t>HOV6</t>
         </is>
       </c>
       <c r="C83" s="235" t="inlineStr">
         <is>
-          <t>WTI Crude</t>
+          <t>NY Harbor ULSD</t>
         </is>
       </c>
       <c r="E83" s="264" t="inlineStr">
         <is>
-          <t>leg of every spread</t>
+          <t>leg of HO/CL and the 3:2:1</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="143">
       <c r="A84" s="249" t="inlineStr">
         <is>
-          <t>INSTRUMENT_4</t>
+          <t>INSTRUMENT_3</t>
         </is>
       </c>
       <c r="B84" s="259" t="inlineStr">
         <is>
-          <t>BZV6</t>
+          <t>CLX6</t>
         </is>
       </c>
       <c r="C84" s="235" t="inlineStr">
         <is>
-          <t>Brent Last Day Financial</t>
+          <t>WTI Crude</t>
         </is>
       </c>
       <c r="E84" s="264" t="inlineStr">
         <is>
-          <t>leg B of BZ - CL</t>
+          <t>leg of every spread</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="143">
       <c r="A85" s="249" t="inlineStr">
         <is>
-          <t>INSTRUMENT_5</t>
+          <t>INSTRUMENT_4</t>
         </is>
       </c>
       <c r="B85" s="259" t="inlineStr">
         <is>
-          <t>CL Oct26 - BZ Oct26 Inter-Product</t>
+          <t>BZX6</t>
         </is>
       </c>
       <c r="C85" s="235" t="inlineStr">
         <is>
-          <t>Exchange-listed inter-product</t>
+          <t>Brent Last Day Financial</t>
         </is>
       </c>
       <c r="E85" s="264" t="inlineStr">
         <is>
-          <t>listed comparison</t>
+          <t>leg B of BZ - CL</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="143">
       <c r="A86" s="249" t="inlineStr">
         <is>
+          <t>INSTRUMENT_5</t>
+        </is>
+      </c>
+      <c r="B86" s="259" t="inlineStr">
+        <is>
+          <t>CL Oct26 - BZ Oct26 Inter-Product</t>
+        </is>
+      </c>
+      <c r="C86" s="235" t="inlineStr">
+        <is>
+          <t>Exchange-listed inter-product</t>
+        </is>
+      </c>
+      <c r="E86" s="264" t="inlineStr">
+        <is>
+          <t>listed comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="15" customHeight="1" s="143">
+      <c r="A87" s="249" t="inlineStr">
+        <is>
           <t>INSTRUMENT_6</t>
         </is>
       </c>
-      <c r="B86" s="259" t="inlineStr">
+      <c r="B87" s="259" t="inlineStr">
         <is>
           <t>Oct26 HO-CL Crack</t>
         </is>
       </c>
-      <c r="C86" s="235" t="inlineStr">
+      <c r="C87" s="235" t="inlineStr">
         <is>
           <t>Exchange-listed crack</t>
         </is>
       </c>
-      <c r="E86" s="264" t="inlineStr">
+      <c r="E87" s="264" t="inlineStr">
         <is>
           <t>listed comparison</t>
         </is>
       </c>
     </row>
-    <row r="87"/>
     <row r="88"/>
-    <row r="89" ht="15" customHeight="1" s="143">
-      <c r="A89" s="255" t="inlineStr">
+    <row r="89"/>
+    <row r="90" ht="15" customHeight="1" s="143">
+      <c r="A90" s="255" t="inlineStr">
         <is>
           <t>SPREAD_TABLE_START   -   up to 4 monitored spreads, one buffer each</t>
         </is>
       </c>
-      <c r="B89" s="262" t="n"/>
-      <c r="C89" s="262" t="n"/>
-      <c r="D89" s="262" t="n"/>
-      <c r="E89" s="262" t="n"/>
-      <c r="F89" s="262" t="n"/>
-      <c r="G89" s="262" t="n"/>
-      <c r="H89" s="262" t="n"/>
-      <c r="I89" s="262" t="n"/>
-      <c r="J89" s="262" t="n"/>
-      <c r="K89" s="262" t="n"/>
-    </row>
-    <row r="90" ht="15" customHeight="1" s="143">
-      <c r="A90" s="230" t="inlineStr">
+      <c r="B90" s="262" t="n"/>
+      <c r="C90" s="262" t="n"/>
+      <c r="D90" s="262" t="n"/>
+      <c r="E90" s="262" t="n"/>
+      <c r="F90" s="262" t="n"/>
+      <c r="G90" s="262" t="n"/>
+      <c r="H90" s="262" t="n"/>
+      <c r="I90" s="262" t="n"/>
+      <c r="J90" s="262" t="n"/>
+      <c r="K90" s="262" t="n"/>
+    </row>
+    <row r="91" ht="15" customHeight="1" s="143">
+      <c r="A91" s="230" t="inlineStr">
         <is>
           <t>Leg COMPOSITION (which instruments, and their weights) is defined by the labelled formulas in the MONITOR LEGS block on the hidden Feed sheet. Everything below is hot-reloaded each tick.</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="32.8" customHeight="1" s="143">
-      <c r="A91" s="256" t="inlineStr">
+    <row r="92" ht="32.8" customHeight="1" s="143">
+      <c r="A92" s="256" t="inlineStr">
         <is>
           <t>Slot</t>
         </is>
       </c>
-      <c r="B91" s="256" t="inlineStr">
+      <c r="B92" s="256" t="inlineStr">
         <is>
           <t>Enabled</t>
         </is>
       </c>
-      <c r="C91" s="256" t="inlineStr">
+      <c r="C92" s="256" t="inlineStr">
         <is>
           <t>Display name</t>
         </is>
       </c>
-      <c r="D91" s="256" t="inlineStr">
+      <c r="D92" s="256" t="inlineStr">
         <is>
           <t>Mode</t>
         </is>
       </c>
-      <c r="E91" s="256" t="inlineStr">
+      <c r="E92" s="256" t="inlineStr">
         <is>
           <t>HEDGE_RATIO (beta)</t>
         </is>
       </c>
-      <c r="F91" s="256" t="inlineStr">
+      <c r="F92" s="256" t="inlineStr">
         <is>
           <t>Beta stamped for pair</t>
         </is>
       </c>
-      <c r="G91" s="256" t="inlineStr">
+      <c r="G92" s="256" t="inlineStr">
         <is>
           <t>USD per 1.00 of spread, per lot</t>
         </is>
       </c>
-      <c r="H91" s="256" t="inlineStr">
+      <c r="H92" s="256" t="inlineStr">
         <is>
           <t>Contracts charged commission</t>
         </is>
       </c>
-      <c r="I91" s="256" t="inlineStr">
+      <c r="I92" s="256" t="inlineStr">
         <is>
           <t>Tick size</t>
         </is>
       </c>
-      <c r="J91" s="256" t="inlineStr">
+      <c r="J92" s="256" t="inlineStr">
         <is>
           <t>Decimals</t>
         </is>
       </c>
-      <c r="K91" s="256" t="inlineStr">
+      <c r="K92" s="256" t="inlineStr">
         <is>
           <t>Listed equivalent (cost comparison)</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="15" customHeight="1" s="143">
-      <c r="A92" s="249" t="inlineStr">
-        <is>
-          <t>SPREAD_1</t>
-        </is>
-      </c>
-      <c r="B92" s="257" t="b">
-        <v>1</v>
-      </c>
-      <c r="C92" s="259" t="inlineStr">
-        <is>
-          <t>BZ - CL  (Brent LDF - WTI)</t>
-        </is>
-      </c>
-      <c r="D92" s="257" t="inlineStr">
-        <is>
-          <t>LEGGED</t>
-        </is>
-      </c>
-      <c r="E92" s="265" t="n">
-        <v>1</v>
-      </c>
-      <c r="F92" s="259" t="inlineStr">
-        <is>
-          <t>BZV6 / CLV6, derived 2026-08 (RELATED pair - no fair value, empirical mean only)</t>
-        </is>
-      </c>
-      <c r="G92" s="266" t="n">
-        <v>1000</v>
-      </c>
-      <c r="H92" s="267" t="n">
-        <v>2</v>
-      </c>
-      <c r="I92" s="265" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="J92" s="267" t="n">
-        <v>2</v>
-      </c>
-      <c r="K92" s="238" t="inlineStr">
-        <is>
-          <t>CL Oct26 - BZ Oct26 Inter-Product</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="143">
       <c r="A93" s="249" t="inlineStr">
         <is>
-          <t>SPREAD_2</t>
+          <t>SPREAD_1</t>
         </is>
       </c>
       <c r="B93" s="257" t="b">
@@ -5633,7 +5595,7 @@
       </c>
       <c r="C93" s="259" t="inlineStr">
         <is>
-          <t>HO/CL crack  (ULSD - WTI)</t>
+          <t>BZ - CL  (Brent LDF - WTI)</t>
         </is>
       </c>
       <c r="D93" s="257" t="inlineStr">
@@ -5646,7 +5608,7 @@
       </c>
       <c r="F93" s="259" t="inlineStr">
         <is>
-          <t>HOV6 x42 / CLV6, 1:1 by design (crack, not a fitted beta)</t>
+          <t>BZV6 / CLV6, derived 2026-08 (RELATED pair - no fair value, empirical mean only)</t>
         </is>
       </c>
       <c r="G93" s="266" t="n">
@@ -5663,14 +5625,14 @@
       </c>
       <c r="K93" s="238" t="inlineStr">
         <is>
-          <t>Oct26 HO-CL Crack</t>
+          <t>CL Oct26 - BZ Oct26 Inter-Product</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="143">
       <c r="A94" s="249" t="inlineStr">
         <is>
-          <t>SPREAD_3</t>
+          <t>SPREAD_2</t>
         </is>
       </c>
       <c r="B94" s="257" t="b">
@@ -5678,7 +5640,7 @@
       </c>
       <c r="C94" s="259" t="inlineStr">
         <is>
-          <t>3:2:1 crack  (2RB+1HO-3CL)/3</t>
+          <t>HO/CL crack  (ULSD - WTI)</t>
         </is>
       </c>
       <c r="D94" s="257" t="inlineStr">
@@ -5691,14 +5653,14 @@
       </c>
       <c r="F94" s="259" t="inlineStr">
         <is>
-          <t>RBV6/HOV6/CLV6, structural 3:2:1 - not a fitted beta</t>
+          <t>HOV6 x42 / CLV6, 1:1 by design (crack, not a fitted beta)</t>
         </is>
       </c>
       <c r="G94" s="266" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="H94" s="267" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I94" s="265" t="n">
         <v>0.01</v>
@@ -5708,14 +5670,14 @@
       </c>
       <c r="K94" s="238" t="inlineStr">
         <is>
-          <t>(none listed)</t>
+          <t>Oct26 HO-CL Crack</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="143">
       <c r="A95" s="249" t="inlineStr">
         <is>
-          <t>SPREAD_4</t>
+          <t>SPREAD_3</t>
         </is>
       </c>
       <c r="B95" s="257" t="b">
@@ -5723,12 +5685,12 @@
       </c>
       <c r="C95" s="259" t="inlineStr">
         <is>
-          <t>CL-BZ Inter-Product (listed)</t>
+          <t>3:2:1 crack  (2RB+1HO-3CL)/3</t>
         </is>
       </c>
       <c r="D95" s="257" t="inlineStr">
         <is>
-          <t>LISTED</t>
+          <t>LEGGED</t>
         </is>
       </c>
       <c r="E95" s="265" t="n">
@@ -5736,14 +5698,14 @@
       </c>
       <c r="F95" s="259" t="inlineStr">
         <is>
-          <t>Exchange-listed spread - beta not applicable</t>
+          <t>RBV6/HOV6/CLV6, structural 3:2:1 - not a fitted beta</t>
         </is>
       </c>
       <c r="G95" s="266" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="H95" s="267" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I95" s="265" t="n">
         <v>0.01</v>
@@ -5753,49 +5715,94 @@
       </c>
       <c r="K95" s="238" t="inlineStr">
         <is>
+          <t>(none listed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="15" customHeight="1" s="143">
+      <c r="A96" s="249" t="inlineStr">
+        <is>
+          <t>SPREAD_4</t>
+        </is>
+      </c>
+      <c r="B96" s="257" t="b">
+        <v>1</v>
+      </c>
+      <c r="C96" s="259" t="inlineStr">
+        <is>
+          <t>CL-BZ Inter-Product (listed)</t>
+        </is>
+      </c>
+      <c r="D96" s="257" t="inlineStr">
+        <is>
+          <t>LISTED</t>
+        </is>
+      </c>
+      <c r="E96" s="265" t="n">
+        <v>1</v>
+      </c>
+      <c r="F96" s="259" t="inlineStr">
+        <is>
+          <t>Exchange-listed spread - beta not applicable</t>
+        </is>
+      </c>
+      <c r="G96" s="266" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H96" s="267" t="n">
+        <v>2</v>
+      </c>
+      <c r="I96" s="265" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J96" s="267" t="n">
+        <v>2</v>
+      </c>
+      <c r="K96" s="238" t="inlineStr">
+        <is>
           <t>n/a - this IS the listed spread</t>
         </is>
       </c>
     </row>
-    <row r="96"/>
-    <row r="97" ht="15" customHeight="1" s="143">
-      <c r="A97" s="252" t="inlineStr">
+    <row r="97"/>
+    <row r="98" ht="15" customHeight="1" s="143">
+      <c r="A98" s="252" t="inlineStr">
         <is>
           <t>HEDGE RATIO BELONGS TO THE PAIR. If the instruments change, beta must be re-derived - a stale beta silently redefines the series. Column F stamps what each beta was computed for.</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="15" customHeight="1" s="143">
-      <c r="A98" s="230" t="inlineStr">
-        <is>
-          <t>Contracts charged: BZ-CL and the listed spread are 2 contracts per lot (one per leg); the 3:2:1 crack is 6 (2 RB + 1 HO + 3 CL).</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="143">
       <c r="A99" s="230" t="inlineStr">
         <is>
+          <t>Contracts charged: BZ-CL and the listed spread are 2 contracts per lot (one per leg); the 3:2:1 crack is 6 (2 RB + 1 HO + 3 CL).</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="15" customHeight="1" s="143">
+      <c r="A100" s="230" t="inlineStr">
+        <is>
           <t>USD per 1.00 of spread: NYMEX energy contracts are 1,000 bbl, so one cent of differential is $10 per leg per lot, i.e. $1,000 per 1.00.</t>
         </is>
       </c>
     </row>
-    <row r="100"/>
-    <row r="101" ht="15" customHeight="1" s="143">
-      <c r="A101" s="252" t="inlineStr">
+    <row r="101"/>
+    <row r="102" ht="15" customHeight="1" s="143">
+      <c r="A102" s="252" t="inlineStr">
         <is>
           <t>NOTIONAL_BASIS - read this before changing it:</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="15" customHeight="1" s="143">
-      <c r="A102" s="230" t="inlineStr">
+    <row r="103" ht="15" customHeight="1" s="143">
+      <c r="A103" s="230" t="inlineStr">
         <is>
           <t>A spread is not an outright, so 'notional' has no single meaning. At 1 lot with CL near $60 and BZ-CL near $7.20:  SPREAD_VALUE ~ $7,200, ONE_LEG ~ $60,000, BOTH_LEGS ~ $127,000.</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="15" customHeight="1" s="143">
-      <c r="A103" s="268" t="inlineStr">
+    <row r="104" ht="15" customHeight="1" s="143">
+      <c r="A104" s="268" t="inlineStr">
         <is>
           <t>1% of those is $72, $600 and $1,270. If sigma on this spread turns out to be ~5 cents ($50), only the first is reachable - the others need the spread to travel 12 or 25 sigma, which it will not do. Watch the TP-in-sigma cell on the Dashboard: above about 1 sigma it turns amber.</t>
         </is>
@@ -5893,7 +5900,7 @@
     </row>
     <row r="6" ht="15" customHeight="1" s="143">
       <c r="A6" s="273">
-        <f>Config!$B$81</f>
+        <f>Config!$B$82</f>
         <v/>
       </c>
       <c r="B6" s="274">
@@ -5932,7 +5939,7 @@
     </row>
     <row r="7" ht="15" customHeight="1" s="143">
       <c r="A7" s="273">
-        <f>Config!$B$82</f>
+        <f>Config!$B$83</f>
         <v/>
       </c>
       <c r="B7" s="274">
@@ -5971,7 +5978,7 @@
     </row>
     <row r="8" ht="15" customHeight="1" s="143">
       <c r="A8" s="273">
-        <f>Config!$B$83</f>
+        <f>Config!$B$84</f>
         <v/>
       </c>
       <c r="B8" s="274">
@@ -6010,7 +6017,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" s="143">
       <c r="A9" s="273">
-        <f>Config!$B$84</f>
+        <f>Config!$B$85</f>
         <v/>
       </c>
       <c r="B9" s="274">
@@ -6049,7 +6056,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" s="143">
       <c r="A10" s="273">
-        <f>Config!$B$85</f>
+        <f>Config!$B$86</f>
         <v/>
       </c>
       <c r="B10" s="274">
@@ -6088,7 +6095,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" s="143">
       <c r="A11" s="273">
-        <f>Config!$B$86</f>
+        <f>Config!$B$87</f>
         <v/>
       </c>
       <c r="B11" s="274">

</xml_diff>